<commit_message>
# formation 101: OD
</commit_message>
<xml_diff>
--- a/database/seeds/sources/staff.xlsx
+++ b/database/seeds/sources/staff.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3591" uniqueCount="2147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3647" uniqueCount="2181">
   <si>
     <t xml:space="preserve">ПЧ</t>
   </si>
@@ -11695,6 +11695,140 @@
   </si>
   <si>
     <t xml:space="preserve">Курманова Айгерим Курмановна</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ОД</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Даус Валерий Арнольдович</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Подполковник, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Оперативный дежурный</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Жаманкулов Аскар Нуржанович</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Майор, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Заместитель ОД</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Турсумбаев Бекжан Айтбекович</t>
+  </si>
+  <si>
+    <t xml:space="preserve">старший лейтенант, Помощник ОД</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Кудеринов Дастан Серикович</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Старшина, Специалист водитель</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Тулпар-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ярцев Денис Николаевич</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Майор,Оперативный дежурный</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Тетроев Руслан Сахрабович</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Майор, Заместитель ОД</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Мырзагалиев Жандос Рашитович</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Попов Александр Юрьевич</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Прапорщик, Специалист водитель</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ганиев Пулат Муратович</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Капитан, оперативный дежурный</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ешмухамбетов Ерганат Талбалдиевич</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Майор,Заместитель ОД</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Оспанов Омар Нургалиевич</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Помощник ОД</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Мусике Куан Абдирулы</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Мусин Диас Радиевич</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Майор, Оперативный дежурный</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ахметов Мурат Маратович</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Капитан, Заместитель ОД</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Шанаев Рахимжан Бакытжанович</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Оспанов Самат Куатович</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Младший сержант, Специалист водитель</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Кияткин Антон Павлович</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Подполковник, Заместитель ОД</t>
+  </si>
+  <si>
+    <t xml:space="preserve">410-411</t>
   </si>
 </sst>
 </file>
@@ -11704,7 +11838,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="31">
+  <fonts count="32">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -11908,6 +12042,11 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -12059,7 +12198,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="80">
+  <cellXfs count="82">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -12380,6 +12519,14 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="25" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="31" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0" customBuiltin="false"/>
@@ -12457,7 +12604,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E1007"/>
+  <dimension ref="A1:E1024"/>
   <sheetFormatPr defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="19.45"/>
@@ -25903,6 +26050,261 @@
       </c>
       <c r="E1007" s="76"/>
     </row>
+    <row r="1008" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1008" s="0" t="s">
+        <v>2147</v>
+      </c>
+      <c r="B1008" s="74" t="s">
+        <v>2148</v>
+      </c>
+      <c r="C1008" s="80"/>
+      <c r="D1008" s="81" t="s">
+        <v>2149</v>
+      </c>
+      <c r="E1008" s="80" t="n">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="1009" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1009" s="0" t="s">
+        <v>2147</v>
+      </c>
+      <c r="B1009" s="74" t="s">
+        <v>2150</v>
+      </c>
+      <c r="C1009" s="80"/>
+      <c r="D1009" s="81" t="s">
+        <v>2151</v>
+      </c>
+      <c r="E1009" s="80" t="n">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="1010" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1010" s="0" t="s">
+        <v>2147</v>
+      </c>
+      <c r="B1010" s="74" t="s">
+        <v>2152</v>
+      </c>
+      <c r="C1010" s="74"/>
+      <c r="D1010" s="80" t="s">
+        <v>2153</v>
+      </c>
+      <c r="E1010" s="80" t="n">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="1011" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1011" s="0" t="s">
+        <v>2147</v>
+      </c>
+      <c r="B1011" s="74" t="s">
+        <v>2154</v>
+      </c>
+      <c r="C1011" s="80"/>
+      <c r="D1011" s="80" t="s">
+        <v>2155</v>
+      </c>
+      <c r="E1011" s="80" t="s">
+        <v>2156</v>
+      </c>
+    </row>
+    <row r="1012" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1012" s="0" t="s">
+        <v>2147</v>
+      </c>
+      <c r="B1012" s="74" t="s">
+        <v>2157</v>
+      </c>
+      <c r="C1012" s="80"/>
+      <c r="D1012" s="80" t="s">
+        <v>2158</v>
+      </c>
+      <c r="E1012" s="80" t="n">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="1013" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1013" s="0" t="s">
+        <v>2147</v>
+      </c>
+      <c r="B1013" s="74" t="s">
+        <v>2159</v>
+      </c>
+      <c r="C1013" s="80"/>
+      <c r="D1013" s="80" t="s">
+        <v>2160</v>
+      </c>
+      <c r="E1013" s="80" t="n">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="1014" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1014" s="0" t="s">
+        <v>2147</v>
+      </c>
+      <c r="B1014" s="74" t="s">
+        <v>2161</v>
+      </c>
+      <c r="C1014" s="80"/>
+      <c r="D1014" s="80" t="s">
+        <v>2153</v>
+      </c>
+      <c r="E1014" s="80" t="n">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="1015" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1015" s="0" t="s">
+        <v>2147</v>
+      </c>
+      <c r="B1015" s="74" t="s">
+        <v>2162</v>
+      </c>
+      <c r="C1015" s="80"/>
+      <c r="D1015" s="80" t="s">
+        <v>2163</v>
+      </c>
+      <c r="E1015" s="80" t="s">
+        <v>2156</v>
+      </c>
+    </row>
+    <row r="1016" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1016" s="0" t="s">
+        <v>2147</v>
+      </c>
+      <c r="B1016" s="74" t="s">
+        <v>2164</v>
+      </c>
+      <c r="C1016" s="80"/>
+      <c r="D1016" s="80" t="s">
+        <v>2165</v>
+      </c>
+      <c r="E1016" s="80" t="n">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="1017" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1017" s="0" t="s">
+        <v>2147</v>
+      </c>
+      <c r="B1017" s="74" t="s">
+        <v>2166</v>
+      </c>
+      <c r="C1017" s="80"/>
+      <c r="D1017" s="80" t="s">
+        <v>2167</v>
+      </c>
+      <c r="E1017" s="80" t="n">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="1018" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1018" s="0" t="s">
+        <v>2147</v>
+      </c>
+      <c r="B1018" s="74" t="s">
+        <v>2168</v>
+      </c>
+      <c r="C1018" s="80"/>
+      <c r="D1018" s="80" t="s">
+        <v>2169</v>
+      </c>
+      <c r="E1018" s="80" t="n">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="1019" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1019" s="0" t="s">
+        <v>2147</v>
+      </c>
+      <c r="B1019" s="74" t="s">
+        <v>2170</v>
+      </c>
+      <c r="C1019" s="80"/>
+      <c r="D1019" s="80" t="s">
+        <v>2155</v>
+      </c>
+      <c r="E1019" s="80" t="s">
+        <v>2156</v>
+      </c>
+    </row>
+    <row r="1020" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1020" s="0" t="s">
+        <v>2147</v>
+      </c>
+      <c r="B1020" s="74" t="s">
+        <v>2171</v>
+      </c>
+      <c r="C1020" s="80"/>
+      <c r="D1020" s="80" t="s">
+        <v>2172</v>
+      </c>
+      <c r="E1020" s="80" t="n">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="1021" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1021" s="0" t="s">
+        <v>2147</v>
+      </c>
+      <c r="B1021" s="74" t="s">
+        <v>2173</v>
+      </c>
+      <c r="C1021" s="80"/>
+      <c r="D1021" s="80" t="s">
+        <v>2174</v>
+      </c>
+      <c r="E1021" s="80" t="n">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="1022" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1022" s="0" t="s">
+        <v>2147</v>
+      </c>
+      <c r="B1022" s="74" t="s">
+        <v>2175</v>
+      </c>
+      <c r="C1022" s="80"/>
+      <c r="D1022" s="80" t="s">
+        <v>2153</v>
+      </c>
+      <c r="E1022" s="80" t="n">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="1023" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1023" s="0" t="s">
+        <v>2147</v>
+      </c>
+      <c r="B1023" s="74" t="s">
+        <v>2176</v>
+      </c>
+      <c r="C1023" s="80"/>
+      <c r="D1023" s="80" t="s">
+        <v>2177</v>
+      </c>
+      <c r="E1023" s="80" t="s">
+        <v>2156</v>
+      </c>
+    </row>
+    <row r="1024" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1024" s="0" t="s">
+        <v>2147</v>
+      </c>
+      <c r="B1024" s="74" t="s">
+        <v>2178</v>
+      </c>
+      <c r="C1024" s="80"/>
+      <c r="D1024" s="80" t="s">
+        <v>2179</v>
+      </c>
+      <c r="E1024" s="80" t="s">
+        <v>2180</v>
+      </c>
+    </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>